<commit_message>
Fix GARANTI POS extraction - correct total 148,190.38 TL
- Extracted from correct HESAP EKSTRESİ section (not product distribution)
- Daily breakdown of Temmuz 2026 transactions
- Grouped by date ranges: 01-10.07, 11-20.07, 21-31.07
- Verified total: 148,190.38 ₺ (matches official TOPLAM)

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013XirDLHEgVkT9Fvb27rTq6
</commit_message>
<xml_diff>
--- a/ISIK_PETROL-GARANTI_POS-Gunluk_Brut-Temmuz2026.xlsx
+++ b/ISIK_PETROL-GARANTI_POS-Gunluk_Brut-Temmuz2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Günlük Brüt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Günlük Brut Tutarlar" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;₺&quot;"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,12 +30,18 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,12 +56,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00366092"/>
+        <bgColor rgb="00366092"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E7E6E6"/>
         <bgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,15 +81,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,314 +482,394 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>AYLIK TOPLAM</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n">
+        <v>148190.38</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Tarih</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Brüt Tutar (TL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>01.07.2026</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>59486.16</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>02.07.2026</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>96247.45199999999</v>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Brüt Tutar</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>03.07.2026</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>102865.03</v>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>01-10.07</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>04.07.2026</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>71232.85000000001</v>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1400</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>05.07.2026</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>176813.71</v>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>3550</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>06.07.2026</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>89146.17</v>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>2150</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>07.07.2026</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>81725.75</v>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>04/07/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>3000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>08.07.2026</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>27004.05</v>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>05/07/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>09.07.2026</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>9177</v>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>4006.45</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>10.07.2026</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>41286</v>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>11.07.2026</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>11987</v>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>8710</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>12.07.2026</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>12088.88</v>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>3650</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>13.07.2026</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>40901</v>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>6450</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>14.07.2026</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>302.31</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>15.07.2026</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>31.78</v>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>01-10.07 TOPLAM</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>35916.45</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>17.07.2026</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>17859</v>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>11-20.07</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>18.07.2026</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>18552</v>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>3139.86</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>19.07.2026</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>39.12</v>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>12/07/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>2612.08</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>20.07.2026</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>61.27</v>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>4210.43</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>21.07.2026</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>139245.6</v>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>1700</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>22.07.2026</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>184066.28</v>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>3400</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>23.07.2026</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>237.23</v>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>6132.389999999999</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>24.07.2026</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>48986</v>
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>4153.32</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>25.07.2026</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>588.5</v>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>19/07/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>246.49</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>26.07.2026</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>26.28</v>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>5390</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>27.07.2026</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>110.27</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>30.07.2026</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>138.3</v>
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>11-20.07 TOPLAM</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>30984.57</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>31.07.2026</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>31306.31</v>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>21-31.07</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>3639.81</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>10419.85</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>7350</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>7700</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>13887.08</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>6759.41</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>2853.34</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>6162.08</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>9177.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>7610.940000000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>5729.75</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>21-31.07 TOPLAM</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n">
+        <v>81289.36</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B30" s="3">
-        <f>SUM(B2:B29)</f>
-        <v/>
+      <c r="B43" s="10" t="n">
+        <v>148190.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>